<commit_message>
MR Angiography Report Codable; client DB copy: --update re-copies a batch of charts, --by-id lists chart ids
- Lab Report > Radiology Report > MR Angiography Report is Codable (taxonomy, copies, page_taxonomy,
  page_canon; APPROACH.md 3.2 table and codeability_review.xlsx).
- clone_client_db.py --update: deletes just the chosen charts from the client DB (matched by chart
  name) and copies our latest; every other chart and all ground truth stay. --by-id: the list file
  holds chart_list ids. --add now skips by chart name. docs/CLIENT_INSTANCE.md 2c.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/codeability_review.xlsx
+++ b/docs/codeability_review.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>MR Angiography Report</t>
+          <t>MRI Report</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3148,7 +3148,7 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>MR Angiography Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
+          <t>MRI Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
         </is>
       </c>
     </row>
@@ -3165,7 +3165,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MRI Report</t>
+          <t>Mammogram Report</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3177,7 +3177,7 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>MRI Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
+          <t>Mammogram Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Mammogram Report</t>
+          <t>Nuclear Medicine Report</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3206,7 +3206,7 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Mammogram Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
+          <t>Nuclear Medicine Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Nuclear Medicine Report</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3235,7 +3235,7 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Nuclear Medicine Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
+          <t>A radiology with no more specific type identified. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Ultrasound Report</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3264,7 +3264,7 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>A radiology with no more specific type identified. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
+          <t>Ultrasound Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Ultrasound Report</t>
+          <t>X-Ray Report</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3293,26 +3293,22 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Ultrasound Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
+          <t>X-Ray Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Lab Report</t>
+          <t>Medication Record</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Radiology Report</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>X-Ray Report</t>
-        </is>
-      </c>
+          <t>Blood Transfusion Record</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
           <t>Non-Codable</t>
@@ -3322,7 +3318,7 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>X-Ray Report. Imaging reports: plain film, CT, MRI, ultrasound, mammography, nuclear medicine, bone density. Angiography is held separately from plain CT and MR because it is a different protocol and a different code.</t>
+          <t>Administration of blood or blood products, which is a medication administration rather than a procedure.</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3330,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Blood Transfusion Record</t>
+          <t>Medication List</t>
         </is>
       </c>
       <c r="C106" t="inlineStr"/>
@@ -3347,7 +3343,7 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Administration of blood or blood products, which is a medication administration rather than a procedure.</t>
+          <t>The current medication list as a standalone page.</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3355,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Medication List</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="C107" t="inlineStr"/>
@@ -3372,7 +3368,7 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>The current medication list as a standalone page.</t>
+          <t>A medication page that fits none of the above.</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3380,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Prescription Page</t>
         </is>
       </c>
       <c r="C108" t="inlineStr"/>
@@ -3397,7 +3393,7 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>A medication page that fits none of the above.</t>
+          <t>A prescription or Rx page.</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3405,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Prescription Page</t>
+          <t>Refill Record</t>
         </is>
       </c>
       <c r="C109" t="inlineStr"/>
@@ -3422,19 +3418,19 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>A prescription or Rx page.</t>
+          <t>A record of refills issued.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Medication Record</t>
+          <t>Order and Requisition</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Refill Record</t>
+          <t>Laboratory Requisition</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
@@ -3447,7 +3443,7 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>A record of refills issued.</t>
+          <t>A requisition or lab form requesting a test.</t>
         </is>
       </c>
     </row>
@@ -3459,7 +3455,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Laboratory Requisition</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
@@ -3472,7 +3468,7 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>A requisition or lab form requesting a test.</t>
+          <t>An order or request that fits neither of the above.</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3480,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Physician Order</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -3497,7 +3493,7 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>An order or request that fits neither of the above.</t>
+          <t>Any order written by a clinician: medication, treatment, service request, post-operative orders.</t>
         </is>
       </c>
     </row>
@@ -3509,7 +3505,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Physician Order</t>
+          <t>Referral Order</t>
         </is>
       </c>
       <c r="C113" t="inlineStr"/>
@@ -3522,19 +3518,19 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Any order written by a clinician: medication, treatment, service request, post-operative orders.</t>
+          <t>Referral Order.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Order and Requisition</t>
+          <t>Patient Communication</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Referral Order</t>
+          <t>Notice</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -3547,7 +3543,7 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Referral Order.</t>
+          <t>A notice or notification sent to the patient, including discharge notices.</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3555,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Notice</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="C115" t="inlineStr"/>
@@ -3572,7 +3568,7 @@
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>A notice or notification sent to the patient, including discharge notices.</t>
+          <t>A communication page that fits none of the above.</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3580,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Patient Education Material</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -3597,7 +3593,7 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>A communication page that fits none of the above.</t>
+          <t>Educational material and patient instructions given out as their own document.</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3605,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Patient Education Material</t>
+          <t>Patient Message</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -3622,7 +3618,7 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Educational material and patient instructions given out as their own document.</t>
+          <t>A message exchanged with the patient: telephone message, portal communication, web encounter.</t>
         </is>
       </c>
     </row>
@@ -3634,7 +3630,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Patient Message</t>
+          <t>Telephone Encounter</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
@@ -3647,19 +3643,19 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>A message exchanged with the patient: telephone message, portal communication, web encounter.</t>
+          <t>Phone note, refill call, telephone message.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Patient Communication</t>
+          <t>Problem List</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Telephone Encounter</t>
+          <t>Diagnosis List/Index</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -3672,7 +3668,7 @@
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Phone note, refill call, telephone message.</t>
+          <t>A list or index of diagnoses, often coded, with no assessment.</t>
         </is>
       </c>
     </row>
@@ -3684,7 +3680,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Diagnosis List/Index</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -3697,7 +3693,7 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>A list or index of diagnoses, often coded, with no assessment.</t>
+          <t>Others.</t>
         </is>
       </c>
     </row>
@@ -3709,7 +3705,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Problem List</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -3722,19 +3718,19 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Others.</t>
+          <t>A standing problem list page.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Problem List</t>
+          <t>Provider Letter</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Problem List</t>
+          <t>Consultation Letter</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -3747,7 +3743,7 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>A standing problem list page.</t>
+          <t>Consultant letter back to the referring provider.</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3755,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Consultation Letter</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
@@ -3772,7 +3768,7 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Consultant letter back to the referring provider.</t>
+          <t>Others.</t>
         </is>
       </c>
     </row>
@@ -3784,7 +3780,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Records Request</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -3797,7 +3793,7 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Others.</t>
+          <t>Any letter, fax or EHR note whose purpose is requesting records.</t>
         </is>
       </c>
     </row>
@@ -3809,7 +3805,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Records Request</t>
+          <t>Referral Letter</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -3822,38 +3818,13 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Any letter, fax or EHR note whose purpose is requesting records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>Provider Letter</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Referral Letter</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr"/>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>Non-Codable</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr">
-        <is>
           <t>Letter referring the patient to another provider.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2 E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E97 E98 E99 E100 E101 E102 E103 E104 E105 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E119 E120 E121 E122 E123 E124 E125 E126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2 E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E97 E98 E99 E100 E101 E102 E103 E104 E105 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E119 E120 E121 E122 E123 E124 E125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Codable,Non-Codable,Discharge"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3867,7 +3838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G168"/>
+  <dimension ref="A1:G167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6731,7 +6702,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MR Angiography Report</t>
+          <t>MR brain report</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -6746,7 +6717,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>MR Angiography Report</t>
+          <t>MRI Report</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -6760,7 +6731,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MR brain report</t>
+          <t>MRI Report</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -6789,7 +6760,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MRI Report</t>
+          <t>Microbiology</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -6799,12 +6770,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Radiology Report</t>
+          <t>Lab Result</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>MRI Report</t>
+          <t>Microbiology Report</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -6818,7 +6789,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Microbiology</t>
+          <t>Microbiology Report</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -6847,7 +6818,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Microbiology Report</t>
+          <t>Mohs surgery report</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -6857,12 +6828,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Lab Result</t>
+          <t>Pathology Report</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Microbiology Report</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -6876,7 +6847,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Mohs surgery report</t>
+          <t>Optical Coherence Tomography Report</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -6886,12 +6857,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Pathology Report</t>
+          <t>Diagnostic Study</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Optical Coherence Tomography Report</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -6905,7 +6876,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Optical Coherence Tomography Report</t>
+          <t>Plethysmography Report</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -6920,7 +6891,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Optical Coherence Tomography Report</t>
+          <t>Plethysmography Report</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -6934,7 +6905,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Plethysmography Report</t>
+          <t>Plethysmography report</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -6963,7 +6934,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Plethysmography report</t>
+          <t>Pulmonary Function Test</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -6978,7 +6949,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Plethysmography Report</t>
+          <t>Pulmonary Function Test</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -6992,7 +6963,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Pulmonary Function Test</t>
+          <t>Pulmonary function test / spirometry</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7021,7 +6992,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Pulmonary function test / spirometry</t>
+          <t>Radiology Report</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -7031,12 +7002,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Diagnostic Study</t>
+          <t>Radiology Report</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Pulmonary Function Test</t>
+          <t>Mammogram Report</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -7050,7 +7021,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Radiology Report</t>
+          <t>Sigmoidoscopy Report</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -7060,12 +7031,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Radiology Report</t>
+          <t>Diagnostic Study</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Mammogram Report</t>
+          <t>Sigmoidoscopy Report</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -7079,7 +7050,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Sigmoidoscopy Report</t>
+          <t>Sonogram Report</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -7089,12 +7060,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Diagnostic Study</t>
+          <t>Radiology Report</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Sigmoidoscopy Report</t>
+          <t>Ultrasound Report</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -7108,7 +7079,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Sonogram Report</t>
+          <t>Sonogram report</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -7137,7 +7108,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Sonogram report</t>
+          <t>Telemetry Report</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -7147,12 +7118,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Radiology Report</t>
+          <t>Diagnostic Study</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Ultrasound Report</t>
+          <t>Telemetry Report</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -7166,7 +7137,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Telemetry Report</t>
+          <t>Tissue Report</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -7176,12 +7147,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Diagnostic Study</t>
+          <t>Pathology Report</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Telemetry Report</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -7195,7 +7166,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Tissue Report</t>
+          <t>Tomography</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -7205,12 +7176,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Pathology Report</t>
+          <t>Radiology Report</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>CT Scan Report</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -7224,7 +7195,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Tomography</t>
+          <t>Tomography Report</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7253,7 +7224,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Tomography Report</t>
+          <t>Ultrasound Report</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7268,7 +7239,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>CT Scan Report</t>
+          <t>Ultrasound Report</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -7282,7 +7253,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Ultrasound Report</t>
+          <t>Urinalysis</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -7292,12 +7263,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Radiology Report</t>
+          <t>Lab Result</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Ultrasound Report</t>
+          <t>Urinalysis Report</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -7311,7 +7282,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Urinalysis</t>
+          <t>Urinalysis Report</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7340,7 +7311,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Urinalysis Report</t>
+          <t>Vascular Studies</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7350,12 +7321,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Lab Result</t>
+          <t>Diagnostic Study</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Urinalysis Report</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -7369,7 +7340,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Vascular Studies</t>
+          <t>X Ray Report</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -7379,12 +7350,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Diagnostic Study</t>
+          <t>Radiology Report</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>X-Ray Report</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -7398,7 +7369,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>X Ray Report</t>
+          <t>X-Ray Report</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -7427,24 +7398,20 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>X-Ray Report</t>
+          <t>Medication List</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Lab Report</t>
+          <t>Medication Record</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Radiology Report</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>X-Ray Report</t>
-        </is>
-      </c>
+          <t>Medication List</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr">
         <is>
           <t>Non-Codable</t>
@@ -7456,7 +7423,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Medication List</t>
+          <t>Medication Reconciliation</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -7481,7 +7448,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Medication Reconciliation</t>
+          <t>Medication Record</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -7489,11 +7456,7 @@
           <t>Medication Record</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>Medication List</t>
-        </is>
-      </c>
+      <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
@@ -7506,15 +7469,19 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
+          <t>Prescription / Rx page</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
           <t>Medication Record</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>Medication Record</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr"/>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Medication List</t>
+        </is>
+      </c>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
@@ -7527,7 +7494,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Prescription / Rx page</t>
+          <t>Prescription Page</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -7537,7 +7504,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Medication List</t>
+          <t>Prescription Page</t>
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
@@ -7552,7 +7519,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Prescription Page</t>
+          <t>Refill Record</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -7562,7 +7529,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Prescription Page</t>
+          <t>Refill Record</t>
         </is>
       </c>
       <c r="D139" t="inlineStr"/>
@@ -7577,7 +7544,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Refill Record</t>
+          <t>Refill record</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -7602,17 +7569,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Refill record</t>
+          <t>Laboratory Requisition</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Medication Record</t>
+          <t>Order and Requisition</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Refill Record</t>
+          <t>Laboratory Requisition</t>
         </is>
       </c>
       <c r="D141" t="inlineStr"/>
@@ -7627,7 +7594,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Laboratory Requisition</t>
+          <t>Medication Orders</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -7637,7 +7604,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Laboratory Requisition</t>
+          <t>Physician Order</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
@@ -7652,7 +7619,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Medication Orders</t>
+          <t>Order and Requisition</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -7660,11 +7627,7 @@
           <t>Order and Requisition</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>Physician Order</t>
-        </is>
-      </c>
+      <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
@@ -7677,15 +7640,19 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
           <t>Order and Requisition</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>Order and Requisition</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr"/>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Physician Order</t>
+        </is>
+      </c>
       <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
@@ -7698,7 +7665,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Orders</t>
+          <t>Physician Order</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -7723,7 +7690,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Physician Order</t>
+          <t>Post Operative Orders</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -7748,7 +7715,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Post Operative Orders</t>
+          <t>Protocols</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -7758,7 +7725,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Physician Order</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
@@ -7773,7 +7740,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Protocols</t>
+          <t>Referral Order</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -7783,7 +7750,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Referral Order</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
@@ -7798,19 +7765,15 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Referral Order</t>
+          <t>Index Page</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Order and Requisition</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Referral Order</t>
-        </is>
-      </c>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
@@ -7823,15 +7786,19 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Index Page</t>
+          <t>General Notice</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Others</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr"/>
+          <t>Patient Communication</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Notice</t>
+        </is>
+      </c>
       <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
@@ -7844,7 +7811,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>General Notice</t>
+          <t>Messages</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -7854,7 +7821,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Notice</t>
+          <t>Patient Message</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
@@ -7869,7 +7836,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Messages</t>
+          <t>Notice</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -7879,7 +7846,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Patient Message</t>
+          <t>Notice</t>
         </is>
       </c>
       <c r="D152" t="inlineStr"/>
@@ -7894,7 +7861,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Notice</t>
+          <t>Notification</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -7904,7 +7871,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Notice</t>
+          <t>Patient Message</t>
         </is>
       </c>
       <c r="D153" t="inlineStr"/>
@@ -7919,7 +7886,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Notification</t>
+          <t>Patient Communication</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -7927,11 +7894,7 @@
           <t>Patient Communication</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Patient Message</t>
-        </is>
-      </c>
+      <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
@@ -7944,15 +7907,19 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
+          <t>Patient Communication &gt; Telephone Encounter</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
           <t>Patient Communication</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>Patient Communication</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr"/>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Telephone Encounter</t>
+        </is>
+      </c>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
@@ -7965,7 +7932,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Patient Communication &gt; Telephone Encounter</t>
+          <t>Patient Education</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -7975,7 +7942,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Telephone Encounter</t>
+          <t>Patient Education Material</t>
         </is>
       </c>
       <c r="D156" t="inlineStr"/>
@@ -7990,7 +7957,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Patient Education</t>
+          <t>Patient Education Material</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -8015,7 +7982,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Patient Education Material</t>
+          <t>Telephone Message</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -8025,7 +7992,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Patient Education Material</t>
+          <t>Patient Message</t>
         </is>
       </c>
       <c r="D158" t="inlineStr"/>
@@ -8040,17 +8007,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Telephone Message</t>
+          <t>Clinical Diagnosis List</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Patient Communication</t>
+          <t>Problem List</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Patient Message</t>
+          <t>Diagnosis List/Index</t>
         </is>
       </c>
       <c r="D159" t="inlineStr"/>
@@ -8065,7 +8032,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Clinical Diagnosis List</t>
+          <t>Problem List</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -8075,7 +8042,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Diagnosis List/Index</t>
+          <t>Problem List</t>
         </is>
       </c>
       <c r="D160" t="inlineStr"/>
@@ -8090,19 +8057,15 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
+          <t>Standalone Patient Summary</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
           <t>Problem List</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Problem List</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Problem List</t>
-        </is>
-      </c>
+      <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
@@ -8115,15 +8078,19 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Standalone Patient Summary</t>
+          <t>Ambulatory Correspondence</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Problem List</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr"/>
+          <t>Provider Letter</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
@@ -8136,7 +8103,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Ambulatory Correspondence</t>
+          <t>Consultation Letter</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -8146,7 +8113,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Consultation Letter</t>
         </is>
       </c>
       <c r="D163" t="inlineStr"/>
@@ -8161,7 +8128,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Consultation Letter</t>
+          <t>Letter</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -8171,7 +8138,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Consultation Letter</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="D164" t="inlineStr"/>
@@ -8186,7 +8153,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Letter</t>
+          <t>Provider Letter (class words)</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -8194,11 +8161,7 @@
           <t>Provider Letter</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
+      <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
@@ -8211,7 +8174,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Provider Letter (class words)</t>
+          <t>Records Request</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -8219,7 +8182,11 @@
           <t>Provider Letter</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr"/>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Records Request</t>
+        </is>
+      </c>
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
@@ -8232,7 +8199,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Records Request</t>
+          <t>Referral Letter</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -8242,7 +8209,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Records Request</t>
+          <t>Referral Letter</t>
         </is>
       </c>
       <c r="D167" t="inlineStr"/>
@@ -8254,34 +8221,9 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr"/>
     </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>Referral Letter</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>Provider Letter</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>Referral Letter</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr"/>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>Non-Codable</t>
-        </is>
-      </c>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41 F42 F43 F44 F45 F46 F47 F48 F49 F50 F51 F52 F53 F54 F55 F56 F57 F58 F59 F60 F61 F62 F63 F64 F65 F66 F67 F68 F69 F70 F71 F72 F73 F74 F75 F76 F77 F78 F79 F80 F81 F82 F83 F84 F85 F86 F87 F88 F89 F90 F91 F92 F93 F94 F95 F96 F97 F98 F99 F100 F101 F102 F103 F104 F105 F106 F107 F108 F109 F110 F111 F112 F113 F114 F115 F116 F117 F118 F119 F120 F121 F122 F123 F124 F125 F126 F127 F128 F129 F130 F131 F132 F133 F134 F135 F136 F137 F138 F139 F140 F141 F142 F143 F144 F145 F146 F147 F148 F149 F150 F151 F152 F153 F154 F155 F156 F157 F158 F159 F160 F161 F162 F163 F164 F165 F166 F167 F168" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3 F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41 F42 F43 F44 F45 F46 F47 F48 F49 F50 F51 F52 F53 F54 F55 F56 F57 F58 F59 F60 F61 F62 F63 F64 F65 F66 F67 F68 F69 F70 F71 F72 F73 F74 F75 F76 F77 F78 F79 F80 F81 F82 F83 F84 F85 F86 F87 F88 F89 F90 F91 F92 F93 F94 F95 F96 F97 F98 F99 F100 F101 F102 F103 F104 F105 F106 F107 F108 F109 F110 F111 F112 F113 F114 F115 F116 F117 F118 F119 F120 F121 F122 F123 F124 F125 F126 F127 F128 F129 F130 F131 F132 F133 F134 F135 F136 F137 F138 F139 F140 F141 F142 F143 F144 F145 F146 F147 F148 F149 F150 F151 F152 F153 F154 F155 F156 F157 F158 F159 F160 F161 F162 F163 F164 F165 F166 F167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Codable,Non-Codable,Discharge"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8295,7 +8237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8357,15 +8299,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Operative Note</t>
+          <t>Lab Report</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anesthesia Record</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>Radiology Report</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MR Angiography Report</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8375,7 +8321,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Critical Care Record</t>
+          <t>Anesthesia Record</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -8388,7 +8334,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Implant Record</t>
+          <t>Critical Care Record</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -8401,7 +8347,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Intra-operative Record</t>
+          <t>Implant Record</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -8414,7 +8360,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Intra-operative Record</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -8427,7 +8373,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Post-operative</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -8440,7 +8386,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pre-operative</t>
+          <t>Post-operative</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -8453,7 +8399,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Procedure List</t>
+          <t>Pre-operative</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -8466,7 +8412,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Surgery Report</t>
+          <t>Procedure List</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -8479,7 +8425,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Triage Report</t>
+          <t>Surgery Report</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -8487,12 +8433,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Procedure Note</t>
+          <t>Operative Note</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cardiac Procedure</t>
+          <t>Triage Report</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -8505,7 +8451,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dialysis Record</t>
+          <t>Cardiac Procedure</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -8518,7 +8464,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Elastography</t>
+          <t>Dialysis Record</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -8531,7 +8477,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Endoscopy (EGD)</t>
+          <t>Elastography</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -8544,7 +8490,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Infusion and Chemotherapy</t>
+          <t>Endoscopy (EGD)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -8557,7 +8503,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Injection Visit</t>
+          <t>Infusion and Chemotherapy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -8570,7 +8516,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Knee Procedure</t>
+          <t>Injection Visit</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -8583,7 +8529,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Laser Procedure</t>
+          <t>Knee Procedure</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -8596,7 +8542,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Lumbar Procedure</t>
+          <t>Laser Procedure</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -8609,7 +8555,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Office Procedure</t>
+          <t>Lumbar Procedure</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -8622,7 +8568,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Office Procedure</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -8635,7 +8581,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pathology Procedure</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -8648,7 +8594,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Radiation Therapy</t>
+          <t>Pathology Procedure</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -8661,7 +8607,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Therapy Session</t>
+          <t>Radiation Therapy</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -8674,7 +8620,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Wound Care</t>
+          <t>Therapy Session</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -8682,12 +8628,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Progress Note</t>
+          <t>Procedure Note</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Assessment and Plan</t>
+          <t>Wound Care</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -8700,7 +8646,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CC/HPI</t>
+          <t>Assessment and Plan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -8713,7 +8659,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Lab and Imaging Results</t>
+          <t>CC/HPI</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -8726,7 +8672,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Medication List</t>
+          <t>Lab and Imaging Results</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -8739,7 +8685,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Others</t>
+          <t>Medication List</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -8752,7 +8698,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Patient Instructions</t>
+          <t>Others</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -8765,7 +8711,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Physical Exam</t>
+          <t>Patient Instructions</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -8778,7 +8724,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Problem List</t>
+          <t>Physical Exam</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -8791,7 +8737,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Procedure List</t>
+          <t>Problem List</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -8804,7 +8750,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Questionnaire</t>
+          <t>Procedure List</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -8817,7 +8763,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Signature</t>
+          <t>Questionnaire</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -8830,7 +8776,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -8843,7 +8789,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Visit Diagnosis</t>
+          <t>Summary</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -8856,10 +8802,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>Visit Diagnosis</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Progress Note</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>Vitals</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>